<commit_message>
Update columns in MCC export
</commit_message>
<xml_diff>
--- a/mcc/resources/web/mcc/exampleData/MCC_Data_Template.xlsx
+++ b/mcc/resources/web/mcc/exampleData/MCC_Data_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\discvr-lk\server\modules\BimberLabKeyModules\mcc\resources\web\mcc\exampleData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7E568A-E233-4563-A200-AAD42BC15A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6191ABD2-1D7D-43E9-B6B4-78BBEC22CDC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="51">
   <si>
     <t>last weight in grams of the animal that was measured</t>
   </si>
@@ -184,6 +184,12 @@
   </si>
   <si>
     <t>Either: 'naïve animal', or 'animal assigned to invasive study'</t>
+  </si>
+  <si>
+    <t>Usage (Current)</t>
+  </si>
+  <si>
+    <t>Usage (Future)</t>
   </si>
 </sst>
 </file>
@@ -246,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -282,9 +288,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -304,12 +307,147 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="28">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="ArialMT"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="ArialMT"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="ArialMT"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="#,##0.0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -328,133 +466,6 @@
       </font>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="ArialMT"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="#,##0.0"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="ArialMT"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <name val="ArialMT"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -469,10 +480,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A7:C25" totalsRowShown="0" headerRowDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A7:C25" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A7:C25" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Minimal Data" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Minimal Data" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="type"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="description"/>
   </tableColumns>
@@ -481,30 +492,32 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{290608B5-1D77-4D67-AB2E-40D153767151}" name="Table2" displayName="Table2" ref="A1:V17" totalsRowShown="0" headerRowDxfId="10" dataDxfId="11">
-  <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{4BC5E10F-3481-4177-B840-6BD64D1CD850}" name="MCC ID" dataDxfId="23"/>
-    <tableColumn id="16" xr3:uid="{93142731-F468-41D6-87E6-6580A09259A5}" name="Center Id" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{2920438D-7068-47F9-9F64-D047DB6E2EC7}" name="Previous IDs" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{FBAEDC2B-AA28-48E9-AD04-616DEC411D5C}" name="Current Colony" dataDxfId="21"/>
-    <tableColumn id="17" xr3:uid="{0ED7CDEE-04EF-4CBB-B811-50391791F255}" name="Source Colony" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{897A3B9D-6380-4B50-8C9E-58EC8ACA2720}" name="Sex" dataDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{2D3904EB-BAB7-4B17-9411-162E98107FAD}" name="Birth" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{507DD53B-06AE-4F42-BECE-BDC6F8A5487F}" name="Status" dataDxfId="20"/>
-    <tableColumn id="22" xr3:uid="{E22BE514-6C88-4F73-A53F-76DB1C711C80}" name="Shipping Destination" dataDxfId="1"/>
-    <tableColumn id="21" xr3:uid="{4BCCE967-6927-43CD-B08D-3203E0044B25}" name="Shipping Date" dataDxfId="2"/>
-    <tableColumn id="20" xr3:uid="{DD8B27DA-161B-44F1-B052-941FF2563DE2}" name="Death" dataDxfId="3"/>
-    <tableColumn id="19" xr3:uid="{3145EA27-CDCE-4A9B-AD1D-BDE857B0B8EA}" name="Cause of Death" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{2401D202-6A40-454E-934B-ADAE25E3CF43}" name="Maternal ID" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{315FCAA6-CCF3-4A2F-BECD-FA25BE79F09B}" name="Paternal ID" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{905FF433-9A5A-4E35-96F2-48082D62D6FE}" name="Weight (g)" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{E3745D04-2DAA-4125-9ABA-78DDD2B99E77}" name="Date of Weight" dataDxfId="16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{290608B5-1D77-4D67-AB2E-40D153767151}" name="Table2" displayName="Table2" ref="A1:X17" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+  <tableColumns count="24">
+    <tableColumn id="1" xr3:uid="{4BC5E10F-3481-4177-B840-6BD64D1CD850}" name="MCC ID" dataDxfId="25"/>
+    <tableColumn id="16" xr3:uid="{93142731-F468-41D6-87E6-6580A09259A5}" name="Center Id" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{2920438D-7068-47F9-9F64-D047DB6E2EC7}" name="Previous IDs" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{FBAEDC2B-AA28-48E9-AD04-616DEC411D5C}" name="Current Colony" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{0ED7CDEE-04EF-4CBB-B811-50391791F255}" name="Source Colony" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{897A3B9D-6380-4B50-8C9E-58EC8ACA2720}" name="Sex" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{2D3904EB-BAB7-4B17-9411-162E98107FAD}" name="Birth" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{507DD53B-06AE-4F42-BECE-BDC6F8A5487F}" name="Status" dataDxfId="18"/>
+    <tableColumn id="22" xr3:uid="{E22BE514-6C88-4F73-A53F-76DB1C711C80}" name="Shipping Destination" dataDxfId="17"/>
+    <tableColumn id="21" xr3:uid="{4BCCE967-6927-43CD-B08D-3203E0044B25}" name="Shipping Date" dataDxfId="16"/>
+    <tableColumn id="20" xr3:uid="{DD8B27DA-161B-44F1-B052-941FF2563DE2}" name="Death" dataDxfId="15"/>
+    <tableColumn id="19" xr3:uid="{3145EA27-CDCE-4A9B-AD1D-BDE857B0B8EA}" name="Cause of Death" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{2401D202-6A40-454E-934B-ADAE25E3CF43}" name="Maternal ID" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{315FCAA6-CCF3-4A2F-BECD-FA25BE79F09B}" name="Paternal ID" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{905FF433-9A5A-4E35-96F2-48082D62D6FE}" name="Weight (g)" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{E3745D04-2DAA-4125-9ABA-78DDD2B99E77}" name="Date of Weight" dataDxfId="10"/>
     <tableColumn id="10" xr3:uid="{1236765E-2035-4367-B5CF-07D96EC7D45D}" name="U24 Status" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{082544F1-788B-4C89-A46D-90592821928D}" name="Availability" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{ED480D88-C3CD-4535-B069-3918904874BC}" name="Current Housing Status" dataDxfId="14"/>
-    <tableColumn id="13" xr3:uid="{42DADF70-CC56-4DC0-8B88-0DC78B97CF61}" name="Infant History" dataDxfId="13"/>
-    <tableColumn id="14" xr3:uid="{188C6861-8A31-4147-ACC0-8B74F64CBE53}" name="Fertility Status" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{082544F1-788B-4C89-A46D-90592821928D}" name="Availability" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{ED480D88-C3CD-4535-B069-3918904874BC}" name="Current Housing Status" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{42DADF70-CC56-4DC0-8B88-0DC78B97CF61}" name="Infant History" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{188C6861-8A31-4147-ACC0-8B74F64CBE53}" name="Fertility Status" dataDxfId="5"/>
     <tableColumn id="25" xr3:uid="{A5D80913-3F77-4B18-B013-3F61B0A2585B}" name="Medical History" dataDxfId="0"/>
+    <tableColumn id="23" xr3:uid="{BA1C546C-36AA-44F6-9C08-872789F17A65}" name="Usage (Current)" dataDxfId="1"/>
+    <tableColumn id="15" xr3:uid="{41E83CCD-834A-49F2-B0D6-8E25976FDC57}" name="Usage (Future)" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -815,11 +828,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
     </row>
     <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="11" t="s">
@@ -836,59 +849,59 @@
       <c r="A8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="15" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="14" t="s">
         <v>14</v>
       </c>
       <c r="B13" t="s">
@@ -899,7 +912,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="14" t="s">
         <v>20</v>
       </c>
       <c r="B14" t="s">
@@ -910,7 +923,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>27</v>
       </c>
       <c r="B15" t="s">
@@ -921,7 +934,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="14" t="s">
         <v>28</v>
       </c>
       <c r="B16" t="s">
@@ -932,7 +945,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="14" t="s">
         <v>29</v>
       </c>
       <c r="B17" t="s">
@@ -943,7 +956,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="14" t="s">
         <v>30</v>
       </c>
       <c r="B18" t="s">
@@ -954,7 +967,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="14" t="s">
         <v>31</v>
       </c>
       <c r="B19" t="s">
@@ -965,7 +978,7 @@
       </c>
     </row>
     <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="14" t="s">
         <v>32</v>
       </c>
       <c r="B20" t="s">
@@ -976,7 +989,7 @@
       </c>
     </row>
     <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B21" t="s">
@@ -987,7 +1000,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="14" t="s">
         <v>34</v>
       </c>
       <c r="B22" t="s">
@@ -998,7 +1011,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="14" t="s">
         <v>35</v>
       </c>
       <c r="B23" t="s">
@@ -1009,7 +1022,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="14" t="s">
         <v>36</v>
       </c>
       <c r="B24" t="s">
@@ -1020,7 +1033,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1">
-      <c r="A25" s="15"/>
+      <c r="A25" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1035,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:X33"/>
+  <dimension ref="A1:Z33"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="13.109375" style="1" customWidth="1"/>
@@ -1048,92 +1061,98 @@
     <col min="18" max="18" width="32.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="19.88671875" style="2" customWidth="1"/>
     <col min="20" max="20" width="22.6640625" style="2" customWidth="1"/>
-    <col min="21" max="22" width="23" style="2" customWidth="1"/>
-    <col min="23" max="23" width="15.21875" customWidth="1"/>
-    <col min="24" max="24" width="19.77734375" customWidth="1"/>
+    <col min="21" max="24" width="23" style="2" customWidth="1"/>
+    <col min="25" max="25" width="15.21875" customWidth="1"/>
+    <col min="26" max="26" width="19.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="9" customFormat="1" ht="31.5">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:25" s="9" customFormat="1" ht="31.5">
+      <c r="A1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="19" t="s">
+      <c r="J1" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="K1" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="19" t="s">
+      <c r="L1" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="N1" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="20" t="s">
+      <c r="O1" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="Q1" s="17" t="s">
+      <c r="Q1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="R1" s="21" t="s">
+      <c r="R1" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="S1" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="21" t="s">
+      <c r="T1" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="U1" s="21" t="s">
+      <c r="U1" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="V1" s="21" t="s">
+      <c r="V1" s="20" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="W1" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="X1" s="20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
       <c r="O2" s="7"/>
@@ -1144,20 +1163,22 @@
       <c r="T2" s="8"/>
       <c r="U2" s="8"/>
       <c r="V2" s="10"/>
-    </row>
-    <row r="3" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+    </row>
+    <row r="3" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
       <c r="F3" s="1"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
       <c r="O3" s="7"/>
@@ -1168,20 +1189,22 @@
       <c r="T3" s="8"/>
       <c r="U3" s="8"/>
       <c r="V3" s="10"/>
-    </row>
-    <row r="4" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
+      <c r="W3" s="8"/>
+      <c r="X3" s="8"/>
+    </row>
+    <row r="4" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="7"/>
@@ -1192,20 +1215,22 @@
       <c r="T4" s="8"/>
       <c r="U4" s="8"/>
       <c r="V4" s="10"/>
-    </row>
-    <row r="5" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="8"/>
+    </row>
+    <row r="5" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="7"/>
@@ -1216,20 +1241,22 @@
       <c r="T5" s="8"/>
       <c r="U5" s="8"/>
       <c r="V5" s="10"/>
-    </row>
-    <row r="6" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+      <c r="W5" s="8"/>
+      <c r="X5" s="8"/>
+    </row>
+    <row r="6" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="7"/>
@@ -1240,20 +1267,22 @@
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
       <c r="V6" s="10"/>
-    </row>
-    <row r="7" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
+      <c r="W6" s="8"/>
+      <c r="X6" s="8"/>
+    </row>
+    <row r="7" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="7"/>
@@ -1264,20 +1293,22 @@
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
       <c r="V7" s="10"/>
-    </row>
-    <row r="8" spans="1:23" s="9" customFormat="1" ht="15.75">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
+      <c r="W7" s="8"/>
+      <c r="X7" s="8"/>
+    </row>
+    <row r="8" spans="1:25" s="9" customFormat="1" ht="15.75">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
       <c r="O8" s="7"/>
@@ -1288,138 +1319,140 @@
       <c r="T8" s="8"/>
       <c r="U8" s="8"/>
       <c r="V8" s="10"/>
-    </row>
-    <row r="9" spans="1:23" ht="15.75">
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
+    </row>
+    <row r="9" spans="1:25" ht="15.75">
       <c r="G9" s="3"/>
       <c r="M9" s="1"/>
       <c r="O9" s="4"/>
       <c r="P9" s="3"/>
-      <c r="Q9" s="18"/>
+      <c r="Q9" s="17"/>
       <c r="R9" s="2"/>
       <c r="V9" s="10"/>
     </row>
-    <row r="10" spans="1:23" ht="15.75">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="G10" s="3"/>
       <c r="M10" s="1"/>
       <c r="O10" s="4"/>
       <c r="P10" s="3"/>
-      <c r="Q10" s="18"/>
+      <c r="Q10" s="17"/>
       <c r="R10" s="2"/>
       <c r="V10" s="10"/>
-      <c r="W10" s="2"/>
-    </row>
-    <row r="11" spans="1:23" ht="15.75">
+      <c r="Y10" s="2"/>
+    </row>
+    <row r="11" spans="1:25" ht="15.75">
       <c r="G11" s="3"/>
       <c r="M11" s="1"/>
       <c r="O11" s="4"/>
       <c r="P11" s="3"/>
-      <c r="Q11" s="18"/>
+      <c r="Q11" s="17"/>
       <c r="R11" s="2"/>
       <c r="V11" s="10"/>
-      <c r="W11" s="2"/>
-    </row>
-    <row r="12" spans="1:23" ht="15.75">
+      <c r="Y11" s="2"/>
+    </row>
+    <row r="12" spans="1:25" ht="15.75">
       <c r="G12" s="3"/>
       <c r="M12" s="1"/>
       <c r="O12" s="4"/>
       <c r="P12" s="3"/>
-      <c r="Q12" s="18"/>
+      <c r="Q12" s="17"/>
       <c r="R12" s="2"/>
       <c r="V12" s="10"/>
-      <c r="W12" s="2"/>
-    </row>
-    <row r="13" spans="1:23" ht="15.75">
+      <c r="Y12" s="2"/>
+    </row>
+    <row r="13" spans="1:25" ht="15.75">
       <c r="G13" s="3"/>
       <c r="M13" s="1"/>
       <c r="O13" s="4"/>
       <c r="P13" s="3"/>
-      <c r="Q13" s="18"/>
+      <c r="Q13" s="17"/>
       <c r="R13" s="2"/>
       <c r="V13" s="10"/>
-      <c r="W13" s="2"/>
-    </row>
-    <row r="14" spans="1:23" ht="15.75">
+      <c r="Y13" s="2"/>
+    </row>
+    <row r="14" spans="1:25" ht="15.75">
       <c r="G14" s="3"/>
       <c r="M14" s="1"/>
       <c r="O14" s="4"/>
       <c r="P14" s="3"/>
-      <c r="Q14" s="18"/>
+      <c r="Q14" s="17"/>
       <c r="R14" s="2"/>
       <c r="V14" s="10"/>
-      <c r="W14" s="2"/>
-    </row>
-    <row r="15" spans="1:23" ht="15.75">
+      <c r="Y14" s="2"/>
+    </row>
+    <row r="15" spans="1:25" ht="15.75">
       <c r="G15" s="3"/>
       <c r="M15" s="1"/>
       <c r="O15" s="4"/>
       <c r="P15" s="3"/>
-      <c r="Q15" s="18"/>
+      <c r="Q15" s="17"/>
       <c r="R15" s="2"/>
       <c r="V15" s="10"/>
-      <c r="W15" s="2"/>
-    </row>
-    <row r="16" spans="1:23" ht="15.75">
+      <c r="Y15" s="2"/>
+    </row>
+    <row r="16" spans="1:25" ht="15.75">
       <c r="G16" s="3"/>
       <c r="M16" s="1"/>
       <c r="O16" s="4"/>
       <c r="P16" s="3"/>
-      <c r="Q16" s="18"/>
+      <c r="Q16" s="17"/>
       <c r="R16" s="2"/>
       <c r="V16" s="10"/>
-      <c r="W16" s="2"/>
-    </row>
-    <row r="17" spans="7:24" ht="15.75">
+      <c r="Y16" s="2"/>
+    </row>
+    <row r="17" spans="7:26" ht="15.75">
       <c r="G17" s="3"/>
       <c r="M17" s="1"/>
       <c r="O17" s="4"/>
       <c r="P17" s="3"/>
-      <c r="Q17" s="18"/>
+      <c r="Q17" s="17"/>
       <c r="R17" s="2"/>
       <c r="V17" s="10"/>
-      <c r="W17" s="2"/>
-    </row>
-    <row r="18" spans="7:24">
-      <c r="W18" s="2"/>
-    </row>
-    <row r="19" spans="7:24">
+      <c r="Y17" s="2"/>
+    </row>
+    <row r="18" spans="7:26">
+      <c r="Y18" s="2"/>
+    </row>
+    <row r="19" spans="7:26">
       <c r="N19" s="13"/>
       <c r="O19" s="13"/>
-      <c r="W19" s="2"/>
-    </row>
-    <row r="20" spans="7:24">
+      <c r="Y19" s="2"/>
+    </row>
+    <row r="20" spans="7:26">
       <c r="N20" s="13"/>
       <c r="O20" s="13"/>
-      <c r="W20" s="2"/>
-    </row>
-    <row r="21" spans="7:24">
+      <c r="Y20" s="2"/>
+    </row>
+    <row r="21" spans="7:26">
       <c r="N21" s="13"/>
       <c r="O21" s="13"/>
     </row>
-    <row r="22" spans="7:24">
+    <row r="22" spans="7:26">
       <c r="N22" s="13"/>
       <c r="O22" s="13"/>
     </row>
-    <row r="23" spans="7:24">
+    <row r="23" spans="7:26">
       <c r="N23" s="13"/>
       <c r="O23" s="13"/>
     </row>
-    <row r="24" spans="7:24">
+    <row r="24" spans="7:26">
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
     </row>
-    <row r="25" spans="7:24">
+    <row r="25" spans="7:26">
       <c r="N25" s="13"/>
       <c r="O25" s="13"/>
     </row>
-    <row r="26" spans="7:24">
+    <row r="26" spans="7:26">
       <c r="N26" s="13"/>
       <c r="O26" s="13"/>
     </row>
-    <row r="28" spans="7:24">
-      <c r="X28" s="2"/>
-    </row>
-    <row r="29" spans="7:24">
-      <c r="X29" s="2"/>
+    <row r="28" spans="7:26">
+      <c r="Z28" s="2"/>
+    </row>
+    <row r="29" spans="7:26">
+      <c r="Z29" s="2"/>
     </row>
     <row r="33" spans="8:12">
       <c r="H33" s="12"/>
@@ -1429,7 +1462,7 @@
       <c r="L33" s="12"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R18:R1048576 Q2:Q17" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"not assigned to U24 breeding colony, assigned to U24 breeding colong"</formula1>
     </dataValidation>
@@ -1439,20 +1472,23 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T18:T1048576 S2:S17" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"singly housed, natal family group, active breeding, social non breeding"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T17 U18:U1048576" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T17 U18:W1048576" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>"no experience, sibling experience only, non successful offspring, successful rearing of offspring"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:U17" xr:uid="{00000000-0002-0000-0100-000005000000}">
-      <formula1>"no mating opportunity, mated no offspring produced, successful offspring produced, hormonal birth control, sterilized"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V1048576" xr:uid="{00000000-0002-0000-0100-000006000000}">
-      <formula1>"naive animal, animal assigned to invasive study"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"male, female"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9:L1048576" xr:uid="{0D74C082-434B-40D3-9E12-118B8C51308C}">
       <formula1>"Alive,Dead,Shipped,Unknown"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:V17" xr:uid="{00000000-0002-0000-0100-000005000000}">
+      <formula1>"no mating opportunity, mated no offspring produced, successful offspring produced, hormonal birth control, sterilized"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X18:X1048576 V2:V17" xr:uid="{00000000-0002-0000-0100-000006000000}">
+      <formula1>"naive animal, animal assigned to invasive study"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:X17" xr:uid="{87A44709-594C-4508-B501-E1D324BD40FD}">
+      <formula1>"breeding, experiment, TBD, other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>